<commit_message>
Add indexed colour test cases to TExcelLayoutTests
</commit_message>
<xml_diff>
--- a/Tests/Samples/Excel/excel.xlsx
+++ b/Tests/Samples/Excel/excel.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64C851DD-1715-45A4-8838-6F565FD4A840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A83BFE-C5F1-4905-8AFE-D4CCE1674132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,12 +30,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
   <si>
     <t>Hello</t>
   </si>
   <si>
     <t>Test</t>
+  </si>
+  <si>
+    <t>Indexed</t>
   </si>
 </sst>
 </file>
@@ -184,7 +187,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -374,6 +377,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="13"/>
       </patternFill>
     </fill>
   </fills>
@@ -537,9 +545,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1019,30 +1030,35 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{594CFBF3-29E5-4614-A58D-8D50B28DA25F}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2">
+      <c r="B1" s="3">
         <v>42</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="3"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
+      <c r="A3" s="4"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
+      <c r="A4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Add column width read and preserve tests to TExcelLayoutTests
</commit_message>
<xml_diff>
--- a/Tests/Samples/Excel/excel.xlsx
+++ b/Tests/Samples/Excel/excel.xlsx
@@ -1032,6 +1032,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{594CFBF3-29E5-4614-A58D-8D50B28DA25F}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>